<commit_message>
Regenerate study_calendar.xlsx with the reading-guide column
The workbook was open in Excel when the reading column was added, so the binary
lagged the generator by one commit. This is the regenerated file: 7 columns
including "מדריך קריאה", ✓ column moved to G with the progress formulas
re-pointed accordingly.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/schedule/study_calendar.xlsx
+++ b/schedule/study_calendar.xlsx
@@ -1269,11 +1269,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1288,7 +1289,7 @@
         </is>
       </c>
       <c r="C1" s="9">
-        <f>COUNTIF(F4:F147,"✓")</f>
+        <f>COUNTIF(G4:G147,"✓")</f>
         <v/>
       </c>
       <c r="D1" s="9" t="inlineStr">
@@ -1338,6 +1339,11 @@
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
+          <t>מדריך קריאה (עמודים בספרים)</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
           <t>הושלם</t>
         </is>
       </c>
@@ -1364,7 +1370,12 @@
       <c r="E4" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F4" s="11" t="inlineStr"/>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 1+4+5, עמ' 3-16, 59-90</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="11" t="n">
@@ -1388,7 +1399,13 @@
       <c r="E5" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="11" t="inlineStr"/>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 6, עמ' 91-106
+Stahl Essential: פרק 1, עמ' 1-28</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="11" t="n">
@@ -1412,7 +1429,12 @@
       <c r="E6" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="11" t="inlineStr"/>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>Stahl Essential: פרק 1+2, עמ' 1-50</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="11" t="n">
@@ -1436,7 +1458,12 @@
       <c r="E7" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="11" t="inlineStr"/>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>Stahl Essential: פרק 4, עמ' 77-158</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="11" t="n">
@@ -1460,7 +1487,12 @@
       <c r="E8" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F8" s="11" t="inlineStr"/>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>Stahl Essential: פרק 5, עמ' 159-243</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="11" t="n">
@@ -1484,7 +1516,12 @@
       <c r="E9" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F9" s="11" t="inlineStr"/>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>Stahl Essential: פרק 6, עמ' 244-282</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="11" t="n">
@@ -1508,7 +1545,12 @@
       <c r="E10" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="11" t="inlineStr"/>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Stahl Essential: פרק 3+6, עמ' 51-76, 244-282</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="11" t="n">
@@ -1532,7 +1574,12 @@
       <c r="E11" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="11" t="inlineStr"/>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 2, עמ' 17-38</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="11" t="n">
@@ -1556,7 +1603,12 @@
       <c r="E12" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="11" t="inlineStr"/>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 3, עמ' 39-58</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="11" t="n">
@@ -1580,7 +1632,12 @@
       <c r="E13" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F13" s="11" t="inlineStr"/>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 4, עמ' 59-74</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="11" t="n">
@@ -1604,7 +1661,12 @@
       <c r="E14" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="11" t="inlineStr"/>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 5, עמ' 75-90</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="11" t="n">
@@ -1628,7 +1690,14 @@
       <c r="E15" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="11" t="inlineStr"/>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 2, עמ' 17-38
+Synopsis: פרק 32
+ℹ תיאוריה — מהכרטיסיות ומ-Synopsis; אין פרק ייעודי ב-Dulcan</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="11" t="n">
@@ -1652,7 +1721,13 @@
       <c r="E16" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F16" s="11" t="inlineStr"/>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Synopsis: פרק 32
+ℹ תיאוריה — מהכרטיסיות ומ-Synopsis; אין פרק ייעודי ב-Dulcan</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="11" t="n">
@@ -1676,7 +1751,13 @@
       <c r="E17" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F17" s="11" t="inlineStr"/>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>DSM-5-TR: Personality Disorders, עמ' 733-778
+Synopsis: פרק 19</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="11" t="n">
@@ -1700,7 +1781,12 @@
       <c r="E18" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F18" s="11" t="inlineStr"/>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 1, עמ' 3-16</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="11" t="n">
@@ -1724,7 +1810,12 @@
       <c r="E19" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F19" s="11" t="inlineStr"/>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 33, עמ' 677-694</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="11" t="n">
@@ -1748,7 +1839,14 @@
       <c r="E20" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F20" s="11" t="inlineStr"/>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 10, עמ' 173-196
+DSM-5-TR: Neurodevelopmental, עמ' 35-100
+Stahl Essential: פרק 11, עמ' 449-485</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="11" t="n">
@@ -1772,7 +1870,14 @@
       <c r="E21" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F21" s="11" t="inlineStr"/>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 34, עמ' 695-728
+Stahl Essential: פרק 11, עמ' 449-485
+Stahl C&amp;A: amphetamine-d, amphetamine-d,l, lisdexamfetamine, methylphenidate-d, methylphenidate-d,l (עמ' 1-36, 269-284, 313-350)</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="11" t="n">
@@ -1796,7 +1901,14 @@
       <c r="E22" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F22" s="11" t="inlineStr"/>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 34, עמ' 695-728
+Stahl Essential: פרק 11, עמ' 449-485
+Stahl C&amp;A: atomoxetine, clonidine, guanfacine, bupropion (עמ' 69-96, 141-154, 243-254)</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="11" t="n">
@@ -1820,7 +1932,13 @@
       <c r="E23" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="F23" s="11" t="inlineStr"/>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 8, עמ' 135-156
+DSM-5-TR: Neurodevelopmental, עמ' 35-100</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="11" t="n">
@@ -1844,7 +1962,13 @@
       <c r="E24" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F24" s="11" t="inlineStr"/>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 7, עמ' 107-134
+DSM-5-TR: Neurodevelopmental, עמ' 35-100</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="11" t="n">
@@ -1868,7 +1992,13 @@
       <c r="E25" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F25" s="11" t="inlineStr"/>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 9, עמ' 157-172
+DSM-5-TR: Neurodevelopmental, עמ' 35-100</t>
+        </is>
+      </c>
+      <c r="G25" s="11" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="n">
@@ -1892,7 +2022,13 @@
       <c r="E26" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F26" s="11" t="inlineStr"/>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 9, עמ' 157-172
+DSM-5-TR: Neurodevelopmental, עמ' 35-100</t>
+        </is>
+      </c>
+      <c r="G26" s="11" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="11" t="n">
@@ -1916,7 +2052,13 @@
       <c r="E27" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F27" s="11" t="inlineStr"/>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 20, עמ' 437-456
+DSM-5-TR: Neurodevelopmental, עמ' 35-100</t>
+        </is>
+      </c>
+      <c r="G27" s="11" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="11" t="n">
@@ -1940,7 +2082,13 @@
       <c r="E28" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F28" s="11" t="inlineStr"/>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 9, עמ' 157-172
+DSM-5-TR: Neurodevelopmental, עמ' 35-100</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="11" t="n">
@@ -1964,7 +2112,12 @@
       <c r="E29" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F29" s="11" t="inlineStr"/>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 7, עמ' 107-134</t>
+        </is>
+      </c>
+      <c r="G29" s="11" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="11" t="n">
@@ -1988,7 +2141,12 @@
       <c r="E30" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F30" s="11" t="inlineStr"/>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 7+8, עמ' 107-156</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="11" t="n">
@@ -2012,7 +2170,14 @@
       <c r="E31" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F31" s="11" t="inlineStr"/>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 13, עמ' 245-278
+DSM-5-TR: Depressive, עמ' 177-214
+Stahl Essential: פרק 6+7, עמ' 244-358</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="11" t="n">
@@ -2036,7 +2201,14 @@
       <c r="E32" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F32" s="11" t="inlineStr"/>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 35, עמ' 729-762
+Stahl Essential: פרק 7, עמ' 283-358
+Stahl C&amp;A: citalopram, escitalopram, fluoxetine, fluvoxamine, paroxetine, sertraline (עמ' 111-124, 185-214, 229-242, 381-396, 439-452)</t>
+        </is>
+      </c>
+      <c r="G32" s="11" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="11" t="n">
@@ -2060,7 +2232,14 @@
       <c r="E33" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="F33" s="11" t="inlineStr"/>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 35, עמ' 729-762
+Stahl Essential: פרק 7, עמ' 283-358
+Stahl C&amp;A: duloxetine, venlafaxine, bupropion, trazodone (עמ' 83-96, 171-184, 453-464, 479-492)</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="11" t="n">
@@ -2084,7 +2263,14 @@
       <c r="E34" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F34" s="11" t="inlineStr"/>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 35, עמ' 729-762
+Stahl Essential: פרק 7, עמ' 283-358
+Stahl C&amp;A: clomipramine (עמ' 125-140)</t>
+        </is>
+      </c>
+      <c r="G34" s="11" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="11" t="n">
@@ -2108,7 +2294,13 @@
       <c r="E35" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F35" s="11" t="inlineStr"/>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 13, עמ' 245-278
+DSM-5-TR: Depressive, עמ' 177-214</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="11" t="n">
@@ -2132,7 +2324,14 @@
       <c r="E36" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F36" s="11" t="inlineStr"/>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 14, עמ' 279-308
+DSM-5-TR: Bipolar, עמ' 139-176
+Stahl Essential: פרק 6+7, עמ' 244-358</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="11" t="n">
@@ -2156,7 +2355,13 @@
       <c r="E37" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F37" s="11" t="inlineStr"/>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 14, עמ' 279-308
+DSM-5-TR: Bipolar, עמ' 139-176</t>
+        </is>
+      </c>
+      <c r="G37" s="11" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="11" t="n">
@@ -2180,7 +2385,14 @@
       <c r="E38" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F38" s="11" t="inlineStr"/>
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 36, עמ' 763-784
+Stahl Essential: פרק 7, עמ' 283-358
+Stahl C&amp;A: lithium (עמ' 285-298)</t>
+        </is>
+      </c>
+      <c r="G38" s="11" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="11" t="n">
@@ -2204,7 +2416,14 @@
       <c r="E39" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F39" s="11" t="inlineStr"/>
+      <c r="F39" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 36, עמ' 763-784
+Stahl Essential: פרק 7, עמ' 283-358
+Stahl C&amp;A: valproate (עמ' 465-478)</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="11" t="n">
@@ -2228,7 +2447,12 @@
       <c r="E40" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F40" s="11" t="inlineStr"/>
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 13+14+26, עמ' 245-308, 551-564</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="11" t="n">
@@ -2252,7 +2476,14 @@
       <c r="E41" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F41" s="11" t="inlineStr"/>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 15, עמ' 309-344
+DSM-5-TR: Anxiety, עמ' 215-262
+Stahl Essential: פרק 8, עמ' 359-378</t>
+        </is>
+      </c>
+      <c r="G41" s="11" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="11" t="n">
@@ -2276,7 +2507,14 @@
       <c r="E42" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F42" s="11" t="inlineStr"/>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 15, עמ' 309-344
+DSM-5-TR: Anxiety, עמ' 215-262
+Stahl Essential: פרק 8, עמ' 359-378</t>
+        </is>
+      </c>
+      <c r="G42" s="11" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="11" t="n">
@@ -2300,7 +2538,13 @@
       <c r="E43" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="F43" s="11" t="inlineStr"/>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 15, עמ' 309-344
+DSM-5-TR: Anxiety, עמ' 215-262</t>
+        </is>
+      </c>
+      <c r="G43" s="11" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="11" t="n">
@@ -2324,7 +2568,13 @@
       <c r="E44" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F44" s="11" t="inlineStr"/>
+      <c r="F44" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 15, עמ' 309-344
+DSM-5-TR: Anxiety, עמ' 215-262</t>
+        </is>
+      </c>
+      <c r="G44" s="11" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="11" t="n">
@@ -2348,7 +2598,12 @@
       <c r="E45" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F45" s="11" t="inlineStr"/>
+      <c r="F45" s="12" t="inlineStr">
+        <is>
+          <t>Stahl Essential: פרק 8+10, עמ' 359-378, 401-448</t>
+        </is>
+      </c>
+      <c r="G45" s="11" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="11" t="n">
@@ -2372,7 +2627,14 @@
       <c r="E46" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F46" s="11" t="inlineStr"/>
+      <c r="F46" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 17, עמ' 365-388
+DSM-5-TR: Obsessive-Compulsive, עמ' 263-294
+Stahl Essential: פרק 13, עמ' 538-578</t>
+        </is>
+      </c>
+      <c r="G46" s="11" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="11" t="n">
@@ -2396,7 +2658,13 @@
       <c r="E47" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F47" s="11" t="inlineStr"/>
+      <c r="F47" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 17+43, עמ' 365-388, 967-984
+Stahl Essential: פרק 13, עמ' 538-578</t>
+        </is>
+      </c>
+      <c r="G47" s="11" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="11" t="n">
@@ -2420,7 +2688,13 @@
       <c r="E48" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F48" s="11" t="inlineStr"/>
+      <c r="F48" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 17, עמ' 365-388
+DSM-5-TR: Obsessive-Compulsive, עמ' 263-294</t>
+        </is>
+      </c>
+      <c r="G48" s="11" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="11" t="n">
@@ -2444,7 +2718,13 @@
       <c r="E49" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F49" s="11" t="inlineStr"/>
+      <c r="F49" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 17, עמ' 365-388
+DSM-5-TR: Obsessive-Compulsive, עמ' 263-294</t>
+        </is>
+      </c>
+      <c r="G49" s="11" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="11" t="n">
@@ -2468,7 +2748,14 @@
       <c r="E50" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F50" s="11" t="inlineStr"/>
+      <c r="F50" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 16, עמ' 345-364
+DSM-5-TR: Trauma, עמ' 295-328
+Stahl Essential: פרק 8, עמ' 359-378</t>
+        </is>
+      </c>
+      <c r="G50" s="11" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="11" t="n">
@@ -2492,7 +2779,13 @@
       <c r="E51" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F51" s="11" t="inlineStr"/>
+      <c r="F51" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 16, עמ' 345-364
+Stahl Essential: פרק 8, עמ' 359-378</t>
+        </is>
+      </c>
+      <c r="G51" s="11" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="11" t="n">
@@ -2516,7 +2809,13 @@
       <c r="E52" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F52" s="11" t="inlineStr"/>
+      <c r="F52" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 16, עמ' 345-364
+DSM-5-TR: Trauma, עמ' 295-328</t>
+        </is>
+      </c>
+      <c r="G52" s="11" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="11" t="n">
@@ -2540,7 +2839,13 @@
       <c r="E53" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F53" s="11" t="inlineStr"/>
+      <c r="F53" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 16, עמ' 345-364
+DSM-5-TR: Trauma, עמ' 295-328</t>
+        </is>
+      </c>
+      <c r="G53" s="11" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="11" t="n">
@@ -2564,7 +2869,12 @@
       <c r="E54" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F54" s="11" t="inlineStr"/>
+      <c r="F54" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 24, עמ' 517-538</t>
+        </is>
+      </c>
+      <c r="G54" s="11" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="11" t="n">
@@ -2588,7 +2898,13 @@
       <c r="E55" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="F55" s="11" t="inlineStr"/>
+      <c r="F55" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 16, עמ' 345-364
+DSM-5-TR: Trauma, עמ' 295-328</t>
+        </is>
+      </c>
+      <c r="G55" s="11" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="11" t="n">
@@ -2612,7 +2928,13 @@
       <c r="E56" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="F56" s="11" t="inlineStr"/>
+      <c r="F56" s="12" t="inlineStr">
+        <is>
+          <t>DSM-5-TR: Dissociative, עמ' 329-348
+Synopsis: פרק 11</t>
+        </is>
+      </c>
+      <c r="G56" s="11" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="11" t="n">
@@ -2636,7 +2958,13 @@
       <c r="E57" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="F57" s="11" t="inlineStr"/>
+      <c r="F57" s="12" t="inlineStr">
+        <is>
+          <t>DSM-5-TR: Somatic Symptom, עמ' 349-370
+Synopsis: פרק 12</t>
+        </is>
+      </c>
+      <c r="G57" s="11" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="11" t="n">
@@ -2660,7 +2988,14 @@
       <c r="E58" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="F58" s="11" t="inlineStr"/>
+      <c r="F58" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 18, עמ' 389-410
+DSM-5-TR: Schizophrenia Spectrum, עמ' 101-138
+Stahl Essential: פרק 4, עמ' 77-158</t>
+        </is>
+      </c>
+      <c r="G58" s="11" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="11" t="n">
@@ -2684,7 +3019,13 @@
       <c r="E59" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="F59" s="11" t="inlineStr"/>
+      <c r="F59" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 18, עמ' 389-410
+Stahl Essential: פרק 4, עמ' 77-158</t>
+        </is>
+      </c>
+      <c r="G59" s="11" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="11" t="n">
@@ -2708,7 +3049,13 @@
       <c r="E60" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="F60" s="11" t="inlineStr"/>
+      <c r="F60" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 18, עמ' 389-410
+DSM-5-TR: Schizophrenia Spectrum, עמ' 101-138</t>
+        </is>
+      </c>
+      <c r="G60" s="11" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="11" t="n">
@@ -2732,7 +3079,14 @@
       <c r="E61" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="F61" s="11" t="inlineStr"/>
+      <c r="F61" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 37, עמ' 785-846
+Stahl Essential: פרק 5, עמ' 159-243
+Stahl C&amp;A: chlorpromazine, fluphenazine, haloperidol, pimozide (עמ' 97-110, 215-228, 255-268, 397-408)</t>
+        </is>
+      </c>
+      <c r="G61" s="11" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="11" t="n">
@@ -2756,7 +3110,14 @@
       <c r="E62" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="F62" s="11" t="inlineStr"/>
+      <c r="F62" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 37, עמ' 785-846
+Stahl Essential: פרק 5, עמ' 159-243
+Stahl C&amp;A: aripiprazole, asenapine, clozapine, lurasidone, olanzapine, paliperidone, quetiapine, risperidone (עמ' 37-68, 155-170, 299-312, 351-380, 409-438)</t>
+        </is>
+      </c>
+      <c r="G62" s="11" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="11" t="n">
@@ -2780,7 +3141,14 @@
       <c r="E63" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="F63" s="11" t="inlineStr"/>
+      <c r="F63" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 37, עמ' 785-846
+Stahl Essential: פרק 5, עמ' 159-243
+Stahl C&amp;A: clozapine (עמ' 155-170)</t>
+        </is>
+      </c>
+      <c r="G63" s="11" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="11" t="n">
@@ -2804,7 +3172,14 @@
       <c r="E64" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="F64" s="11" t="inlineStr"/>
+      <c r="F64" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 37, עמ' 785-846
+Stahl Essential: פרק 5, עמ' 159-243
+Stahl C&amp;A: aripiprazole (עמ' 37-54)</t>
+        </is>
+      </c>
+      <c r="G64" s="11" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="11" t="n">
@@ -2828,7 +3203,14 @@
       <c r="E65" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="F65" s="11" t="inlineStr"/>
+      <c r="F65" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 37, עמ' 785-846
+Stahl Essential: פרק 5, עמ' 159-243
+Stahl C&amp;A: olanzapine, quetiapine, risperidone (עמ' 351-366, 409-438)</t>
+        </is>
+      </c>
+      <c r="G65" s="11" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="11" t="n">
@@ -2852,7 +3234,14 @@
       <c r="E66" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="F66" s="11" t="inlineStr"/>
+      <c r="F66" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 37, עמ' 785-846
+Stahl Essential: פרק 5, עמ' 159-243
+Stahl C&amp;A: lurasidone (עמ' 299-312)</t>
+        </is>
+      </c>
+      <c r="G66" s="11" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="11" t="n">
@@ -2876,7 +3265,14 @@
       <c r="E67" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="F67" s="11" t="inlineStr"/>
+      <c r="F67" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 37, עמ' 785-846
+Stahl Essential: פרק 5, עמ' 159-243
+Stahl C&amp;A: paliperidone, risperidone (עמ' 367-380, 423-438)</t>
+        </is>
+      </c>
+      <c r="G67" s="11" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="11" t="n">
@@ -2900,7 +3296,14 @@
       <c r="E68" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="F68" s="11" t="inlineStr"/>
+      <c r="F68" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 37, עמ' 785-846
+DSM-5-TR: Medication-Induced Movement, עמ' 807-820
+Stahl Essential: פרק 5, עמ' 159-243</t>
+        </is>
+      </c>
+      <c r="G68" s="11" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="11" t="n">
@@ -2924,7 +3327,13 @@
       <c r="E69" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="F69" s="11" t="inlineStr"/>
+      <c r="F69" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 37, עמ' 785-846
+DSM-5-TR: Medication-Induced Movement, עמ' 807-820</t>
+        </is>
+      </c>
+      <c r="G69" s="11" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="11" t="n">
@@ -2948,7 +3357,13 @@
       <c r="E70" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="F70" s="11" t="inlineStr"/>
+      <c r="F70" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 37+29, עמ' 605-620, 785-846
+DSM-5-TR: Medication-Induced Movement, עמ' 807-820</t>
+        </is>
+      </c>
+      <c r="G70" s="11" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="11" t="n">
@@ -2972,7 +3387,12 @@
       <c r="E71" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="F71" s="11" t="inlineStr"/>
+      <c r="F71" s="12" t="inlineStr">
+        <is>
+          <t>DSM-5-TR: Schizophrenia Spectrum, עמ' 101-138</t>
+        </is>
+      </c>
+      <c r="G71" s="11" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="11" t="n">
@@ -2996,7 +3416,12 @@
       <c r="E72" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="F72" s="11" t="inlineStr"/>
+      <c r="F72" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 29, עמ' 605-620</t>
+        </is>
+      </c>
+      <c r="G72" s="11" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="11" t="n">
@@ -3020,7 +3445,13 @@
       <c r="E73" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="F73" s="11" t="inlineStr"/>
+      <c r="F73" s="12" t="inlineStr">
+        <is>
+          <t>Synopsis: פרק 22
+ℹ ECT — Synopsis פרק 22; אין פרק ייעודי ב-Dulcan</t>
+        </is>
+      </c>
+      <c r="G73" s="11" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="11" t="n">
@@ -3044,7 +3475,14 @@
       <c r="E74" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="F74" s="11" t="inlineStr"/>
+      <c r="F74" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 22, עמ' 473-502
+DSM-5-TR: Sleep-Wake, עמ' 407-476
+Stahl Essential: פרק 10, עמ' 401-448</t>
+        </is>
+      </c>
+      <c r="G74" s="11" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="11" t="n">
@@ -3068,7 +3506,13 @@
       <c r="E75" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="F75" s="11" t="inlineStr"/>
+      <c r="F75" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 22, עמ' 473-502
+Stahl Essential: פרק 10, עמ' 401-448</t>
+        </is>
+      </c>
+      <c r="G75" s="11" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="11" t="n">
@@ -3092,7 +3536,14 @@
       <c r="E76" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="F76" s="11" t="inlineStr"/>
+      <c r="F76" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 22, עמ' 473-502
+DSM-5-TR: Sleep-Wake, עמ' 407-476
+Stahl Essential: פרק 10, עמ' 401-448</t>
+        </is>
+      </c>
+      <c r="G76" s="11" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="11" t="n">
@@ -3116,7 +3567,13 @@
       <c r="E77" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="F77" s="11" t="inlineStr"/>
+      <c r="F77" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 22, עמ' 473-502
+DSM-5-TR: Sleep-Wake, עמ' 407-476</t>
+        </is>
+      </c>
+      <c r="G77" s="11" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="11" t="n">
@@ -3140,7 +3597,13 @@
       <c r="E78" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="F78" s="11" t="inlineStr"/>
+      <c r="F78" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 19, עמ' 411-436
+DSM-5-TR: Feeding and Eating, עמ' 371-398</t>
+        </is>
+      </c>
+      <c r="G78" s="11" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="11" t="n">
@@ -3164,7 +3627,13 @@
       <c r="E79" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="F79" s="11" t="inlineStr"/>
+      <c r="F79" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 19, עמ' 411-436
+DSM-5-TR: Feeding and Eating, עמ' 371-398</t>
+        </is>
+      </c>
+      <c r="G79" s="11" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="11" t="n">
@@ -3188,7 +3657,13 @@
       <c r="E80" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="F80" s="11" t="inlineStr"/>
+      <c r="F80" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 19, עמ' 411-436
+DSM-5-TR: Feeding and Eating, עמ' 371-398</t>
+        </is>
+      </c>
+      <c r="G80" s="11" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="11" t="n">
@@ -3212,7 +3687,13 @@
       <c r="E81" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="F81" s="11" t="inlineStr"/>
+      <c r="F81" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 21, עמ' 457-472
+DSM-5-TR: Elimination, עמ' 399-406</t>
+        </is>
+      </c>
+      <c r="G81" s="11" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="11" t="n">
@@ -3236,7 +3717,12 @@
       <c r="E82" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="F82" s="11" t="inlineStr"/>
+      <c r="F82" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 22, עמ' 473-502</t>
+        </is>
+      </c>
+      <c r="G82" s="11" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="11" t="n">
@@ -3260,7 +3746,12 @@
       <c r="E83" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="F83" s="11" t="inlineStr"/>
+      <c r="F83" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 19+41, עמ' 411-436, 933-954</t>
+        </is>
+      </c>
+      <c r="G83" s="11" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="11" t="n">
@@ -3284,7 +3775,13 @@
       <c r="E84" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="F84" s="11" t="inlineStr"/>
+      <c r="F84" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 12, עמ' 221-244
+DSM-5-TR: Substance, עמ' 543-666</t>
+        </is>
+      </c>
+      <c r="G84" s="11" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="11" t="n">
@@ -3308,7 +3805,13 @@
       <c r="E85" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="F85" s="11" t="inlineStr"/>
+      <c r="F85" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 12, עמ' 221-244
+Stahl Essential: פרק 13, עמ' 538-578</t>
+        </is>
+      </c>
+      <c r="G85" s="11" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="11" t="n">
@@ -3332,7 +3835,13 @@
       <c r="E86" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="F86" s="11" t="inlineStr"/>
+      <c r="F86" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 12, עמ' 221-244
+DSM-5-TR: Substance, עמ' 543-666</t>
+        </is>
+      </c>
+      <c r="G86" s="11" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="11" t="n">
@@ -3356,7 +3865,13 @@
       <c r="E87" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="F87" s="11" t="inlineStr"/>
+      <c r="F87" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 12, עמ' 221-244
+Stahl Essential: פרק 13, עמ' 538-578</t>
+        </is>
+      </c>
+      <c r="G87" s="11" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="11" t="n">
@@ -3380,7 +3895,14 @@
       <c r="E88" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="F88" s="11" t="inlineStr"/>
+      <c r="F88" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 12, עמ' 221-244
+DSM-5-TR: Substance, עמ' 543-666
+Stahl Essential: פרק 13, עמ' 538-578</t>
+        </is>
+      </c>
+      <c r="G88" s="11" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="11" t="n">
@@ -3404,7 +3926,13 @@
       <c r="E89" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="F89" s="11" t="inlineStr"/>
+      <c r="F89" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 12, עמ' 221-244
+DSM-5-TR: Substance, עמ' 543-666</t>
+        </is>
+      </c>
+      <c r="G89" s="11" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="11" t="n">
@@ -3428,7 +3956,13 @@
       <c r="E90" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="F90" s="11" t="inlineStr"/>
+      <c r="F90" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 12, עמ' 221-244
+Stahl C&amp;A: bupropion (עמ' 83-96)</t>
+        </is>
+      </c>
+      <c r="G90" s="11" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="11" t="n">
@@ -3452,7 +3986,13 @@
       <c r="E91" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="F91" s="11" t="inlineStr"/>
+      <c r="F91" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 12, עמ' 221-244
+DSM-5-TR: Substance, עמ' 543-666</t>
+        </is>
+      </c>
+      <c r="G91" s="11" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="11" t="n">
@@ -3476,7 +4016,13 @@
       <c r="E92" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="F92" s="11" t="inlineStr"/>
+      <c r="F92" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 12, עמ' 221-244
+DSM-5-TR: Substance, עמ' 543-666</t>
+        </is>
+      </c>
+      <c r="G92" s="11" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="11" t="n">
@@ -3500,7 +4046,14 @@
       <c r="E93" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="F93" s="11" t="inlineStr"/>
+      <c r="F93" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 12, עמ' 221-244
+DSM-5-TR: Substance, עמ' 543-666
+Stahl Essential: פרק 13, עמ' 538-578</t>
+        </is>
+      </c>
+      <c r="G93" s="11" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="11" t="n">
@@ -3524,7 +4077,13 @@
       <c r="E94" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="F94" s="11" t="inlineStr"/>
+      <c r="F94" s="12" t="inlineStr">
+        <is>
+          <t>DSM-5-TR: Personality Disorders, עמ' 733-778
+Synopsis: פרק 19</t>
+        </is>
+      </c>
+      <c r="G94" s="11" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="11" t="n">
@@ -3548,7 +4107,13 @@
       <c r="E95" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="F95" s="11" t="inlineStr"/>
+      <c r="F95" s="12" t="inlineStr">
+        <is>
+          <t>DSM-5-TR: Personality Disorders, עמ' 733-778
+Synopsis: פרק 19</t>
+        </is>
+      </c>
+      <c r="G95" s="11" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="11" t="n">
@@ -3572,7 +4137,13 @@
       <c r="E96" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="F96" s="11" t="inlineStr"/>
+      <c r="F96" s="12" t="inlineStr">
+        <is>
+          <t>DSM-5-TR: Personality Disorders, עמ' 733-778
+Synopsis: פרק 19</t>
+        </is>
+      </c>
+      <c r="G96" s="11" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="11" t="n">
@@ -3596,7 +4167,13 @@
       <c r="E97" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="F97" s="11" t="inlineStr"/>
+      <c r="F97" s="12" t="inlineStr">
+        <is>
+          <t>DSM-5-TR: Personality Disorders, עמ' 733-778
+Synopsis: פרק 19</t>
+        </is>
+      </c>
+      <c r="G97" s="11" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="11" t="n">
@@ -3620,7 +4197,13 @@
       <c r="E98" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="F98" s="11" t="inlineStr"/>
+      <c r="F98" s="12" t="inlineStr">
+        <is>
+          <t>Synopsis: פרק 19, 23
+ℹ טיפול DBT ב-BPD — Synopsis; אין פרק ייעודי ב-Dulcan</t>
+        </is>
+      </c>
+      <c r="G98" s="11" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="11" t="n">
@@ -3644,7 +4227,14 @@
       <c r="E99" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="F99" s="11" t="inlineStr"/>
+      <c r="F99" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 11, עמ' 197-220
+DSM-5-TR: Personality Disorders, עמ' 733-778
+Synopsis: פרק 19</t>
+        </is>
+      </c>
+      <c r="G99" s="11" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="11" t="n">
@@ -3668,7 +4258,13 @@
       <c r="E100" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="F100" s="11" t="inlineStr"/>
+      <c r="F100" s="12" t="inlineStr">
+        <is>
+          <t>DSM-5-TR: Personality Disorders, עמ' 733-778
+Synopsis: פרק 19</t>
+        </is>
+      </c>
+      <c r="G100" s="11" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="11" t="n">
@@ -3692,7 +4288,13 @@
       <c r="E101" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="F101" s="11" t="inlineStr"/>
+      <c r="F101" s="12" t="inlineStr">
+        <is>
+          <t>DSM-5-TR: Personality Disorders, עמ' 733-778
+Synopsis: פרק 19</t>
+        </is>
+      </c>
+      <c r="G101" s="11" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="11" t="n">
@@ -3716,7 +4318,13 @@
       <c r="E102" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="F102" s="11" t="inlineStr"/>
+      <c r="F102" s="12" t="inlineStr">
+        <is>
+          <t>DSM-5-TR: Personality Disorders, עמ' 733-778
+Synopsis: פרק 19</t>
+        </is>
+      </c>
+      <c r="G102" s="11" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="11" t="n">
@@ -3740,7 +4348,13 @@
       <c r="E103" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="F103" s="11" t="inlineStr"/>
+      <c r="F103" s="12" t="inlineStr">
+        <is>
+          <t>DSM-5-TR: Personality Disorders, עמ' 733-778
+Synopsis: פרק 19</t>
+        </is>
+      </c>
+      <c r="G103" s="11" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="11" t="n">
@@ -3764,7 +4378,13 @@
       <c r="E104" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="F104" s="11" t="inlineStr"/>
+      <c r="F104" s="12" t="inlineStr">
+        <is>
+          <t>DSM-5-TR: Personality Disorders, עמ' 733-778
+Synopsis: פרק 19</t>
+        </is>
+      </c>
+      <c r="G104" s="11" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="11" t="n">
@@ -3788,7 +4408,13 @@
       <c r="E105" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="F105" s="11" t="inlineStr"/>
+      <c r="F105" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 31, עמ' 637-652
+Synopsis: פרק 28</t>
+        </is>
+      </c>
+      <c r="G105" s="11" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="11" t="n">
@@ -3812,7 +4438,13 @@
       <c r="E106" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="F106" s="11" t="inlineStr"/>
+      <c r="F106" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 31, עמ' 637-652
+ℹ הדין הישראלי — חקיקה מקומית; לא מכוסה בספרי הלימוד</t>
+        </is>
+      </c>
+      <c r="G106" s="11" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="11" t="n">
@@ -3836,7 +4468,13 @@
       <c r="E107" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="F107" s="11" t="inlineStr"/>
+      <c r="F107" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 27, עמ' 565-580
+DSM-5-TR: Gender Dysphoria, עמ' 511-520</t>
+        </is>
+      </c>
+      <c r="G107" s="11" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="11" t="n">
@@ -3860,7 +4498,13 @@
       <c r="E108" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="F108" s="11" t="inlineStr"/>
+      <c r="F108" s="12" t="inlineStr">
+        <is>
+          <t>DSM-5-TR: Sexual Dysfunctions · Paraphilic, עמ' 477-510, 779-802
+Synopsis: פרק 16</t>
+        </is>
+      </c>
+      <c r="G108" s="11" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="11" t="n">
@@ -3884,7 +4528,13 @@
       <c r="E109" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="F109" s="11" t="inlineStr"/>
+      <c r="F109" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 11, עמ' 197-220
+DSM-5-TR: Disruptive, עמ' 521-542</t>
+        </is>
+      </c>
+      <c r="G109" s="11" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="11" t="n">
@@ -3908,7 +4558,12 @@
       <c r="E110" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="F110" s="11" t="inlineStr"/>
+      <c r="F110" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 28, עמ' 581-604</t>
+        </is>
+      </c>
+      <c r="G110" s="11" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="11" t="n">
@@ -3932,7 +4587,12 @@
       <c r="E111" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="F111" s="11" t="inlineStr"/>
+      <c r="F111" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 26, עמ' 551-564</t>
+        </is>
+      </c>
+      <c r="G111" s="11" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="11" t="n">
@@ -3956,7 +4616,12 @@
       <c r="E112" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="F112" s="11" t="inlineStr"/>
+      <c r="F112" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 26, עמ' 551-564</t>
+        </is>
+      </c>
+      <c r="G112" s="11" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="11" t="n">
@@ -3980,7 +4645,12 @@
       <c r="E113" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="F113" s="11" t="inlineStr"/>
+      <c r="F113" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 30, עמ' 621-636</t>
+        </is>
+      </c>
+      <c r="G113" s="11" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="11" t="n">
@@ -4004,7 +4674,12 @@
       <c r="E114" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="F114" s="11" t="inlineStr"/>
+      <c r="F114" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 25, עמ' 539-550</t>
+        </is>
+      </c>
+      <c r="G114" s="11" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="11" t="n">
@@ -4028,7 +4703,13 @@
       <c r="E115" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="F115" s="11" t="inlineStr"/>
+      <c r="F115" s="12" t="inlineStr">
+        <is>
+          <t>DSM-5-TR: Depressive, עמ' 177-214
+ℹ פסיכיאטריה פרינטלית — specifier peripartum ב-DSM; הרחבה בכרטיסיות</t>
+        </is>
+      </c>
+      <c r="G115" s="11" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="11" t="n">
@@ -4052,7 +4733,12 @@
       <c r="E116" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="F116" s="11" t="inlineStr"/>
+      <c r="F116" s="12" t="inlineStr">
+        <is>
+          <t>Stahl Essential: פרק 7, עמ' 283-358</t>
+        </is>
+      </c>
+      <c r="G116" s="11" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="11" t="n">
@@ -4076,7 +4762,14 @@
       <c r="E117" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="F117" s="11" t="inlineStr"/>
+      <c r="F117" s="12" t="inlineStr">
+        <is>
+          <t>DSM-5-TR: Neurocognitive, עמ' 667-732
+Stahl Essential: פרק 12, עמ' 486-537
+Synopsis: פרק 3</t>
+        </is>
+      </c>
+      <c r="G117" s="11" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="11" t="n">
@@ -4100,7 +4793,13 @@
       <c r="E118" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="F118" s="11" t="inlineStr"/>
+      <c r="F118" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 6, עמ' 91-106
+Stahl Essential: פרק 1, עמ' 1-28</t>
+        </is>
+      </c>
+      <c r="G118" s="11" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="11" t="n">
@@ -4124,7 +4823,12 @@
       <c r="E119" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="F119" s="11" t="inlineStr"/>
+      <c r="F119" s="12" t="inlineStr">
+        <is>
+          <t>ℹ נוירולוגיה — מהסילבוס ומהכרטיסיות; אין פרק ייעודי בספרי הליבה</t>
+        </is>
+      </c>
+      <c r="G119" s="11" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="11" t="n">
@@ -4148,7 +4852,12 @@
       <c r="E120" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="F120" s="11" t="inlineStr"/>
+      <c r="F120" s="12" t="inlineStr">
+        <is>
+          <t>ℹ נוירולוגיה — מהסילבוס ומהכרטיסיות; אין פרק ייעודי בספרי הליבה</t>
+        </is>
+      </c>
+      <c r="G120" s="11" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="11" t="n">
@@ -4172,7 +4881,12 @@
       <c r="E121" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="F121" s="11" t="inlineStr"/>
+      <c r="F121" s="12" t="inlineStr">
+        <is>
+          <t>ℹ נוירולוגיה — מהסילבוס ומהכרטיסיות; אין פרק ייעודי בספרי הליבה</t>
+        </is>
+      </c>
+      <c r="G121" s="11" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="11" t="n">
@@ -4196,7 +4910,12 @@
       <c r="E122" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="F122" s="11" t="inlineStr"/>
+      <c r="F122" s="12" t="inlineStr">
+        <is>
+          <t>ℹ נוירולוגיה — מהסילבוס ומהכרטיסיות; אין פרק ייעודי בספרי הליבה</t>
+        </is>
+      </c>
+      <c r="G122" s="11" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="11" t="n">
@@ -4220,7 +4939,12 @@
       <c r="E123" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="F123" s="11" t="inlineStr"/>
+      <c r="F123" s="12" t="inlineStr">
+        <is>
+          <t>ℹ נוירולוגיה — מהסילבוס ומהכרטיסיות; אין פרק ייעודי בספרי הליבה</t>
+        </is>
+      </c>
+      <c r="G123" s="11" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="11" t="n">
@@ -4244,7 +4968,12 @@
       <c r="E124" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="F124" s="11" t="inlineStr"/>
+      <c r="F124" s="12" t="inlineStr">
+        <is>
+          <t>ℹ נוירולוגיה — מהסילבוס ומהכרטיסיות; אין פרק ייעודי בספרי הליבה</t>
+        </is>
+      </c>
+      <c r="G124" s="11" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="11" t="n">
@@ -4268,7 +4997,13 @@
       <c r="E125" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="F125" s="11" t="inlineStr"/>
+      <c r="F125" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 7+8, עמ' 107-156
+ℹ סינדרומים נוירוגנטיים — Dulcan 7-8 + הסילבוס</t>
+        </is>
+      </c>
+      <c r="G125" s="11" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="11" t="n">
@@ -4292,7 +5027,13 @@
       <c r="E126" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="F126" s="11" t="inlineStr"/>
+      <c r="F126" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 7, עמ' 107-134
+ℹ נוירוקוטנאיים — Dulcan 7 + הסילבוס</t>
+        </is>
+      </c>
+      <c r="G126" s="11" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="11" t="n">
@@ -4316,7 +5057,12 @@
       <c r="E127" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="F127" s="11" t="inlineStr"/>
+      <c r="F127" s="12" t="inlineStr">
+        <is>
+          <t>ℹ נוירולוגיה — מהסילבוס ומהכרטיסיות; אין פרק ייעודי בספרי הליבה</t>
+        </is>
+      </c>
+      <c r="G127" s="11" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="11" t="n">
@@ -4340,7 +5086,12 @@
       <c r="E128" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="F128" s="11" t="inlineStr"/>
+      <c r="F128" s="12" t="inlineStr">
+        <is>
+          <t>ℹ נוירולוגיה — מהסילבוס ומהכרטיסיות; אין פרק ייעודי בספרי הליבה</t>
+        </is>
+      </c>
+      <c r="G128" s="11" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="11" t="n">
@@ -4364,7 +5115,12 @@
       <c r="E129" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="F129" s="11" t="inlineStr"/>
+      <c r="F129" s="12" t="inlineStr">
+        <is>
+          <t>ℹ נוירולוגיה — מהסילבוס ומהכרטיסיות; אין פרק ייעודי בספרי הליבה</t>
+        </is>
+      </c>
+      <c r="G129" s="11" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="11" t="n">
@@ -4388,7 +5144,12 @@
       <c r="E130" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="F130" s="11" t="inlineStr"/>
+      <c r="F130" s="12" t="inlineStr">
+        <is>
+          <t>ℹ נוירולוגיה — מהסילבוס ומהכרטיסיות; אין פרק ייעודי בספרי הליבה</t>
+        </is>
+      </c>
+      <c r="G130" s="11" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="11" t="n">
@@ -4412,7 +5173,13 @@
       <c r="E131" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="F131" s="11" t="inlineStr"/>
+      <c r="F131" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 22, עמ' 473-502
+Stahl Essential: פרק 10, עמ' 401-448</t>
+        </is>
+      </c>
+      <c r="G131" s="11" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="11" t="n">
@@ -4436,7 +5203,12 @@
       <c r="E132" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="F132" s="11" t="inlineStr"/>
+      <c r="F132" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 29, עמ' 605-620</t>
+        </is>
+      </c>
+      <c r="G132" s="11" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="11" t="n">
@@ -4460,7 +5232,12 @@
       <c r="E133" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="F133" s="11" t="inlineStr"/>
+      <c r="F133" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 48+49, עמ' 1071-1161</t>
+        </is>
+      </c>
+      <c r="G133" s="11" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="11" t="n">
@@ -4484,7 +5261,13 @@
       <c r="E134" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="F134" s="11" t="inlineStr"/>
+      <c r="F134" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 38, עמ' 847-872
+Synopsis: פרק 23</t>
+        </is>
+      </c>
+      <c r="G134" s="11" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="11" t="n">
@@ -4508,7 +5291,13 @@
       <c r="E135" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="F135" s="11" t="inlineStr"/>
+      <c r="F135" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 43, עמ' 967-984
+Synopsis: פרק 23</t>
+        </is>
+      </c>
+      <c r="G135" s="11" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="11" t="n">
@@ -4532,7 +5321,13 @@
       <c r="E136" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="F136" s="11" t="inlineStr"/>
+      <c r="F136" s="12" t="inlineStr">
+        <is>
+          <t>Synopsis: פרק 23
+ℹ DBT — Synopsis פרק 23; אין פרק ייעודי ב-Dulcan</t>
+        </is>
+      </c>
+      <c r="G136" s="11" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="11" t="n">
@@ -4556,7 +5351,12 @@
       <c r="E137" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="F137" s="11" t="inlineStr"/>
+      <c r="F137" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 42, עמ' 955-966</t>
+        </is>
+      </c>
+      <c r="G137" s="11" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="11" t="n">
@@ -4580,7 +5380,12 @@
       <c r="E138" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="F138" s="11" t="inlineStr"/>
+      <c r="F138" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 44, עמ' 985-998</t>
+        </is>
+      </c>
+      <c r="G138" s="11" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="11" t="n">
@@ -4604,7 +5409,12 @@
       <c r="E139" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="F139" s="11" t="inlineStr"/>
+      <c r="F139" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 45+46, עמ' 999-1042</t>
+        </is>
+      </c>
+      <c r="G139" s="11" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="11" t="n">
@@ -4628,7 +5438,12 @@
       <c r="E140" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="F140" s="11" t="inlineStr"/>
+      <c r="F140" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 47, עמ' 1043-1070</t>
+        </is>
+      </c>
+      <c r="G140" s="11" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="11" t="n">
@@ -4652,7 +5467,12 @@
       <c r="E141" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="F141" s="11" t="inlineStr"/>
+      <c r="F141" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 40+41, עמ' 899-954</t>
+        </is>
+      </c>
+      <c r="G141" s="11" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="11" t="n">
@@ -4676,7 +5496,13 @@
       <c r="E142" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="F142" s="11" t="inlineStr"/>
+      <c r="F142" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 38, עמ' 847-872
+Synopsis: פרק 23</t>
+        </is>
+      </c>
+      <c r="G142" s="11" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="11" t="n">
@@ -4700,7 +5526,14 @@
       <c r="E143" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="F143" s="11" t="inlineStr"/>
+      <c r="F143" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 38, עמ' 847-872
+Synopsis: פרק 23
+ℹ תיאוריה — מהכרטיסיות ומ-Synopsis; אין פרק ייעודי ב-Dulcan</t>
+        </is>
+      </c>
+      <c r="G143" s="11" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="11" t="n">
@@ -4724,7 +5557,13 @@
       <c r="E144" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="F144" s="11" t="inlineStr"/>
+      <c r="F144" s="12" t="inlineStr">
+        <is>
+          <t>Synopsis: פרק 23
+ℹ תיאוריה — מהכרטיסיות ומ-Synopsis; אין פרק ייעודי ב-Dulcan</t>
+        </is>
+      </c>
+      <c r="G144" s="11" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="11" t="n">
@@ -4748,7 +5587,12 @@
       <c r="E145" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="F145" s="11" t="inlineStr"/>
+      <c r="F145" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 32, עמ' 653-676</t>
+        </is>
+      </c>
+      <c r="G145" s="11" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="11" t="n">
@@ -4772,7 +5616,12 @@
       <c r="E146" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="F146" s="11" t="inlineStr"/>
+      <c r="F146" s="12" t="inlineStr">
+        <is>
+          <t>Dulcan: פרק 23, עמ' 503-516</t>
+        </is>
+      </c>
+      <c r="G146" s="11" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="11" t="n">
@@ -4796,11 +5645,16 @@
       <c r="E147" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="F147" s="11" t="inlineStr"/>
+      <c r="F147" s="12" t="inlineStr">
+        <is>
+          <t>ℹ סקירת אינטגרציה — כל החומר</t>
+        </is>
+      </c>
+      <c r="G147" s="11" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F4:F147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G4:G147" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"✓,"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>